<commit_message>
Update Excel date parsing and enhance admin UI components
- Improved date parsing logic in `import-legacy-from-xlsx.ts` to handle various date formats, including Buddhist Era years and Excel serial dates, ensuring accurate date storage.
- Enhanced CSS styles in `admin.css` for better dropdown menu handling and improved layout consistency in the admin interface.
- Updated `MemberReviewSummary.tsx` to reflect more descriptive section titles for member details and contact information.
- Modified `DashboardPage.tsx` to include a new class for panels with dropdowns, enhancing the user experience in the admin dashboard.

These changes improve the accuracy of date handling and enhance the overall usability of the admin interface.
</commit_message>
<xml_diff>
--- a/ABTA-System/Data/NewMemDatabase.xlsx
+++ b/ABTA-System/Data/NewMemDatabase.xlsx
@@ -8,7 +8,7 @@
       <x15ac:absPath xmlns:x15ac="http://schemas.microsoft.com/office/spreadsheetml/2010/11/ac" url="D:\Work\Fastwork\Customer\ABTA\ABTA-System\Data\"/>
     </mc:Choice>
   </mc:AlternateContent>
-  <xr:revisionPtr revIDLastSave="0" documentId="13_ncr:1_{96F78743-A70F-4FC3-8ACD-A02ABA709F9B}" xr6:coauthVersionLast="47" xr6:coauthVersionMax="47" xr10:uidLastSave="{00000000-0000-0000-0000-000000000000}"/>
+  <xr:revisionPtr revIDLastSave="0" documentId="13_ncr:1_{AB4E73D2-D457-43A7-8C33-4308C9BEE163}" xr6:coauthVersionLast="47" xr6:coauthVersionMax="47" xr10:uidLastSave="{00000000-0000-0000-0000-000000000000}"/>
   <bookViews>
     <workbookView xWindow="-120" yWindow="-120" windowWidth="29040" windowHeight="15720" activeTab="1" xr2:uid="{4E62CD03-FB27-40C9-B490-48A30120C3FE}"/>
   </bookViews>
@@ -40,7 +40,7 @@
 </file>
 
 <file path=xl/sharedStrings.xml><?xml version="1.0" encoding="utf-8"?>
-<sst xmlns="http://schemas.openxmlformats.org/spreadsheetml/2006/main" count="125" uniqueCount="95">
+<sst xmlns="http://schemas.openxmlformats.org/spreadsheetml/2006/main" count="138" uniqueCount="103">
   <si>
     <t>ที่อยู่อีเมล</t>
   </si>
@@ -325,6 +325,30 @@
   </si>
   <si>
     <t>จำนวนเงิน</t>
+  </si>
+  <si>
+    <t>Cakepuarknomsod2@gmail.com</t>
+  </si>
+  <si>
+    <t>0808026677</t>
+  </si>
+  <si>
+    <t>3-001</t>
+  </si>
+  <si>
+    <t>PK Residence</t>
+  </si>
+  <si>
+    <t>18/3 ถนนเทศบาล 46 ตำบลวารินชำราบ อำเภอวารินชำราบ จังหวัดอุบลราชธานี 34190</t>
+  </si>
+  <si>
+    <t>เพชญเกล้า จำปารัตน์</t>
+  </si>
+  <si>
+    <t>บุณยาพร อรุนยะเดช</t>
+  </si>
+  <si>
+    <t>M001</t>
   </si>
 </sst>
 </file>
@@ -854,22 +878,22 @@
 
 <file path=xl/worksheets/sheet1.xml><?xml version="1.0" encoding="utf-8"?>
 <worksheet xmlns="http://schemas.openxmlformats.org/spreadsheetml/2006/main" xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" xmlns:mc="http://schemas.openxmlformats.org/markup-compatibility/2006" xmlns:x14ac="http://schemas.microsoft.com/office/spreadsheetml/2009/9/ac" xmlns:xr="http://schemas.microsoft.com/office/spreadsheetml/2014/revision" xmlns:xr2="http://schemas.microsoft.com/office/spreadsheetml/2015/revision2" xmlns:xr3="http://schemas.microsoft.com/office/spreadsheetml/2016/revision3" mc:Ignorable="x14ac xr xr2 xr3" xr:uid="{809A2A7A-CEA4-4090-82B5-AC4F6EF40CF9}">
-  <dimension ref="A1:T6"/>
+  <dimension ref="A1:T7"/>
   <sheetFormatPr defaultRowHeight="15" x14ac:dyDescent="0.25"/>
   <cols>
-    <col min="1" max="1" width="13.42578125" bestFit="1" customWidth="1"/>
-    <col min="2" max="2" width="21.85546875" customWidth="1"/>
-    <col min="3" max="3" width="10.7109375" bestFit="1" customWidth="1"/>
+    <col min="1" max="1" width="15.5703125" bestFit="1" customWidth="1"/>
+    <col min="2" max="2" width="29.85546875" customWidth="1"/>
+    <col min="3" max="3" width="14.85546875" customWidth="1"/>
     <col min="4" max="4" width="25.140625" bestFit="1" customWidth="1"/>
     <col min="5" max="5" width="9.28515625" bestFit="1" customWidth="1"/>
-    <col min="6" max="6" width="14.7109375" bestFit="1" customWidth="1"/>
+    <col min="6" max="6" width="29" customWidth="1"/>
     <col min="7" max="7" width="21" bestFit="1" customWidth="1"/>
-    <col min="8" max="8" width="18.28515625" bestFit="1" customWidth="1"/>
+    <col min="8" max="8" width="74.85546875" customWidth="1"/>
     <col min="9" max="9" width="16" bestFit="1" customWidth="1"/>
-    <col min="10" max="10" width="13.42578125" bestFit="1" customWidth="1"/>
-    <col min="11" max="11" width="16.28515625" bestFit="1" customWidth="1"/>
-    <col min="12" max="12" width="20.28515625" bestFit="1" customWidth="1"/>
-    <col min="13" max="13" width="23.5703125" customWidth="1"/>
+    <col min="10" max="10" width="27.5703125" customWidth="1"/>
+    <col min="11" max="11" width="23.5703125" customWidth="1"/>
+    <col min="12" max="12" width="20.42578125" bestFit="1" customWidth="1"/>
+    <col min="13" max="13" width="66.85546875" customWidth="1"/>
     <col min="14" max="14" width="29.42578125" customWidth="1"/>
     <col min="15" max="15" width="34.42578125" customWidth="1"/>
     <col min="16" max="16" width="69" customWidth="1"/>
@@ -1209,6 +1233,62 @@
         <v>45</v>
       </c>
     </row>
+    <row r="7" spans="1:20" ht="30" x14ac:dyDescent="0.25">
+      <c r="A7" s="3">
+        <v>46224.416666666664</v>
+      </c>
+      <c r="B7" s="15" t="s">
+        <v>95</v>
+      </c>
+      <c r="C7" s="5" t="s">
+        <v>96</v>
+      </c>
+      <c r="D7" s="4" t="s">
+        <v>27</v>
+      </c>
+      <c r="E7" s="4" t="s">
+        <v>97</v>
+      </c>
+      <c r="F7" s="4" t="s">
+        <v>98</v>
+      </c>
+      <c r="G7" s="4">
+        <v>808026677</v>
+      </c>
+      <c r="H7" s="4" t="s">
+        <v>99</v>
+      </c>
+      <c r="I7" s="4" t="s">
+        <v>37</v>
+      </c>
+      <c r="J7" s="4" t="s">
+        <v>100</v>
+      </c>
+      <c r="K7" s="4" t="s">
+        <v>101</v>
+      </c>
+      <c r="L7" s="7">
+        <v>1347600018247</v>
+      </c>
+      <c r="M7" s="4" t="s">
+        <v>99</v>
+      </c>
+      <c r="N7" s="14"/>
+      <c r="O7" s="14"/>
+      <c r="P7" s="14"/>
+      <c r="Q7" s="8" t="b">
+        <v>1</v>
+      </c>
+      <c r="R7" s="9">
+        <v>244551.625</v>
+      </c>
+      <c r="S7" s="9">
+        <v>244551.79166666666</v>
+      </c>
+      <c r="T7" s="4" t="s">
+        <v>45</v>
+      </c>
+    </row>
   </sheetData>
   <hyperlinks>
     <hyperlink ref="B2" r:id="rId1" xr:uid="{03CD33D4-0FC6-4FE6-ACD4-48614D4041E4}"/>
@@ -1216,6 +1296,7 @@
     <hyperlink ref="B4" r:id="rId3" xr:uid="{C2BF0BEE-9E55-4301-96E6-945B48B3E77E}"/>
     <hyperlink ref="B5" r:id="rId4" xr:uid="{5655DBB8-FD38-49A3-9CA2-A44332C1F6CC}"/>
     <hyperlink ref="B6" r:id="rId5" xr:uid="{13E6A275-AA3E-4734-A693-2526E5294827}"/>
+    <hyperlink ref="B7" r:id="rId6" xr:uid="{EC58BA91-01A5-4071-95E8-B2F3E2377B46}"/>
   </hyperlinks>
   <pageMargins left="0.7" right="0.7" top="0.75" bottom="0.75" header="0.3" footer="0.3"/>
 </worksheet>
@@ -1226,7 +1307,7 @@
   <dimension ref="A1:K13"/>
   <sheetFormatPr defaultRowHeight="15" x14ac:dyDescent="0.25"/>
   <cols>
-    <col min="1" max="1" width="14" customWidth="1"/>
+    <col min="1" max="1" width="17.85546875" customWidth="1"/>
     <col min="2" max="2" width="19.85546875" customWidth="1"/>
     <col min="3" max="3" width="20.7109375" customWidth="1"/>
     <col min="4" max="4" width="35.42578125" customWidth="1"/>
@@ -1237,6 +1318,9 @@
     <col min="9" max="9" width="20.85546875" customWidth="1"/>
     <col min="10" max="10" width="16.28515625" customWidth="1"/>
     <col min="11" max="11" width="15.7109375" customWidth="1"/>
+    <col min="12" max="12" width="14.140625" bestFit="1" customWidth="1"/>
+    <col min="18" max="19" width="14.42578125" bestFit="1" customWidth="1"/>
+    <col min="20" max="20" width="27.140625" customWidth="1"/>
   </cols>
   <sheetData>
     <row r="1" spans="1:11" x14ac:dyDescent="0.25">
@@ -1274,7 +1358,7 @@
         <v>19</v>
       </c>
     </row>
-    <row r="2" spans="1:11" ht="39" x14ac:dyDescent="0.25">
+    <row r="2" spans="1:11" x14ac:dyDescent="0.25">
       <c r="A2" s="16" t="s">
         <v>23</v>
       </c>
@@ -1309,7 +1393,7 @@
         <v>1</v>
       </c>
     </row>
-    <row r="3" spans="1:11" ht="51.75" x14ac:dyDescent="0.25">
+    <row r="3" spans="1:11" x14ac:dyDescent="0.25">
       <c r="A3" s="11">
         <v>242091</v>
       </c>
@@ -1344,7 +1428,7 @@
         <v>1</v>
       </c>
     </row>
-    <row r="4" spans="1:11" ht="39" x14ac:dyDescent="0.25">
+    <row r="4" spans="1:11" x14ac:dyDescent="0.25">
       <c r="A4" s="11">
         <v>242093</v>
       </c>
@@ -1414,7 +1498,7 @@
         <v>1</v>
       </c>
     </row>
-    <row r="6" spans="1:11" ht="26.25" x14ac:dyDescent="0.25">
+    <row r="6" spans="1:11" x14ac:dyDescent="0.25">
       <c r="A6" s="11">
         <v>242093</v>
       </c>
@@ -1449,18 +1533,42 @@
         <v>1</v>
       </c>
     </row>
-    <row r="7" spans="1:11" ht="26.25" x14ac:dyDescent="0.25">
+    <row r="7" spans="1:11" x14ac:dyDescent="0.25">
+      <c r="A7" s="11">
+        <v>46224</v>
+      </c>
+      <c r="B7" s="9">
+        <v>46224.416666666664</v>
+      </c>
       <c r="C7" s="19" t="s">
         <v>31</v>
       </c>
-      <c r="D7" s="23" t="s">
+      <c r="D7" s="20" t="s">
         <v>84</v>
       </c>
       <c r="E7" s="22">
         <v>500</v>
       </c>
-    </row>
-    <row r="8" spans="1:11" ht="26.25" x14ac:dyDescent="0.25">
+      <c r="F7" s="4" t="s">
+        <v>97</v>
+      </c>
+      <c r="G7" s="21" t="s">
+        <v>102</v>
+      </c>
+      <c r="H7" s="8" t="b">
+        <v>1</v>
+      </c>
+      <c r="I7" s="9">
+        <v>244551.625</v>
+      </c>
+      <c r="J7" s="10">
+        <v>244714</v>
+      </c>
+      <c r="K7" s="8" t="b">
+        <v>1</v>
+      </c>
+    </row>
+    <row r="8" spans="1:11" x14ac:dyDescent="0.25">
       <c r="C8" s="19" t="s">
         <v>31</v>
       </c>
@@ -1471,7 +1579,7 @@
         <v>5000</v>
       </c>
     </row>
-    <row r="9" spans="1:11" ht="51.75" x14ac:dyDescent="0.25">
+    <row r="9" spans="1:11" x14ac:dyDescent="0.25">
       <c r="C9" s="17" t="s">
         <v>2</v>
       </c>
@@ -1482,7 +1590,7 @@
         <v>500</v>
       </c>
     </row>
-    <row r="10" spans="1:11" ht="51.75" x14ac:dyDescent="0.25">
+    <row r="10" spans="1:11" x14ac:dyDescent="0.25">
       <c r="C10" s="17" t="s">
         <v>2</v>
       </c>
@@ -1493,7 +1601,7 @@
         <v>1000</v>
       </c>
     </row>
-    <row r="11" spans="1:11" ht="26.25" x14ac:dyDescent="0.25">
+    <row r="11" spans="1:11" x14ac:dyDescent="0.25">
       <c r="C11" s="17" t="s">
         <v>87</v>
       </c>
@@ -1504,7 +1612,7 @@
         <v>1000</v>
       </c>
     </row>
-    <row r="12" spans="1:11" ht="26.25" x14ac:dyDescent="0.25">
+    <row r="12" spans="1:11" x14ac:dyDescent="0.25">
       <c r="C12" s="17" t="s">
         <v>87</v>
       </c>
@@ -1515,7 +1623,7 @@
         <v>500</v>
       </c>
     </row>
-    <row r="13" spans="1:11" ht="26.25" x14ac:dyDescent="0.25">
+    <row r="13" spans="1:11" x14ac:dyDescent="0.25">
       <c r="C13" s="17" t="s">
         <v>87</v>
       </c>

</xml_diff>

<commit_message>
Enhance legacy member management and update notification features
- Introduced a new API endpoint for listing legacy members, allowing admin users to browse and search through legacy data.
- Implemented functionality to stage member ID and receipt number changes during data reviews, improving the accuracy of member information.
- Updated the admin interface to include new components for handling ID changes, enhancing user experience during member reviews.
- Enhanced notification logic to inform members about updates to their IDs and receipt numbers, ensuring clear communication.

These changes improve the overall functionality of legacy member management and enhance the user experience in the admin interface.
</commit_message>
<xml_diff>
--- a/ABTA-System/Data/NewMemDatabase.xlsx
+++ b/ABTA-System/Data/NewMemDatabase.xlsx
@@ -8,9 +8,9 @@
       <x15ac:absPath xmlns:x15ac="http://schemas.microsoft.com/office/spreadsheetml/2010/11/ac" url="D:\Work\Fastwork\Customer\ABTA\ABTA-System\Data\"/>
     </mc:Choice>
   </mc:AlternateContent>
-  <xr:revisionPtr revIDLastSave="0" documentId="13_ncr:1_{AB4E73D2-D457-43A7-8C33-4308C9BEE163}" xr6:coauthVersionLast="47" xr6:coauthVersionMax="47" xr10:uidLastSave="{00000000-0000-0000-0000-000000000000}"/>
+  <xr:revisionPtr revIDLastSave="0" documentId="13_ncr:1_{2793354F-CF36-4727-9914-E3FB6C482E68}" xr6:coauthVersionLast="47" xr6:coauthVersionMax="47" xr10:uidLastSave="{00000000-0000-0000-0000-000000000000}"/>
   <bookViews>
-    <workbookView xWindow="-120" yWindow="-120" windowWidth="29040" windowHeight="15720" activeTab="1" xr2:uid="{4E62CD03-FB27-40C9-B490-48A30120C3FE}"/>
+    <workbookView xWindow="7800" yWindow="2760" windowWidth="21600" windowHeight="11835" xr2:uid="{4E62CD03-FB27-40C9-B490-48A30120C3FE}"/>
   </bookViews>
   <sheets>
     <sheet name="Member" sheetId="1" r:id="rId1"/>
@@ -40,7 +40,7 @@
 </file>
 
 <file path=xl/sharedStrings.xml><?xml version="1.0" encoding="utf-8"?>
-<sst xmlns="http://schemas.openxmlformats.org/spreadsheetml/2006/main" count="138" uniqueCount="103">
+<sst xmlns="http://schemas.openxmlformats.org/spreadsheetml/2006/main" count="139" uniqueCount="103">
   <si>
     <t>ที่อยู่อีเมล</t>
   </si>
@@ -965,7 +965,7 @@
         <v>40</v>
       </c>
     </row>
-    <row r="2" spans="1:20" ht="39" x14ac:dyDescent="0.25">
+    <row r="2" spans="1:20" x14ac:dyDescent="0.25">
       <c r="A2" s="3">
         <v>46222.417170833331</v>
       </c>
@@ -1021,7 +1021,7 @@
         <v>45</v>
       </c>
     </row>
-    <row r="3" spans="1:20" ht="39" x14ac:dyDescent="0.25">
+    <row r="3" spans="1:20" x14ac:dyDescent="0.25">
       <c r="A3" s="3">
         <v>46222.417170833331</v>
       </c>
@@ -1075,7 +1075,7 @@
         <v>46</v>
       </c>
     </row>
-    <row r="4" spans="1:20" ht="30" x14ac:dyDescent="0.25">
+    <row r="4" spans="1:20" x14ac:dyDescent="0.25">
       <c r="A4" s="3">
         <v>46222.417170833331</v>
       </c>
@@ -1129,7 +1129,7 @@
         <v>47</v>
       </c>
     </row>
-    <row r="5" spans="1:20" ht="51.75" x14ac:dyDescent="0.25">
+    <row r="5" spans="1:20" x14ac:dyDescent="0.25">
       <c r="A5" s="3">
         <v>46222.417170833331</v>
       </c>
@@ -1179,9 +1179,9 @@
         <v>48</v>
       </c>
     </row>
-    <row r="6" spans="1:20" ht="39" x14ac:dyDescent="0.25">
+    <row r="6" spans="1:20" x14ac:dyDescent="0.25">
       <c r="A6" s="3">
-        <v>46222.417170833331</v>
+        <v>46222.417175925926</v>
       </c>
       <c r="B6" s="15" t="s">
         <v>76</v>
@@ -1252,8 +1252,8 @@
       <c r="F7" s="4" t="s">
         <v>98</v>
       </c>
-      <c r="G7" s="4">
-        <v>808026677</v>
+      <c r="G7" s="5" t="s">
+        <v>96</v>
       </c>
       <c r="H7" s="4" t="s">
         <v>99</v>

</xml_diff>